<commit_message>
project finished, all features implemented
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="108">
   <si>
     <t>UPC</t>
   </si>
@@ -167,12 +167,6 @@
     <t>Acana Healthy Grains Large Breed 10.2kg</t>
   </si>
   <si>
-    <t>UPC000023</t>
-  </si>
-  <si>
-    <t>ACANA Puppy Small Breed Dry Dog Food</t>
-  </si>
-  <si>
     <t>UPC000024</t>
   </si>
   <si>
@@ -326,18 +320,6 @@
     <t>Accessory Cat Grooming Brush</t>
   </si>
   <si>
-    <t>UPC000048</t>
-  </si>
-  <si>
-    <t>Dog Food Mixed Breed Beef &amp; Chicken 10kg</t>
-  </si>
-  <si>
-    <t>UPC000049</t>
-  </si>
-  <si>
-    <t>Cat Food Salmon &amp; Turkey Mixed Dry Food 5kg</t>
-  </si>
-  <si>
     <t>UPC000050</t>
   </si>
   <si>
@@ -347,22 +329,20 @@
     <t>UPC000051</t>
   </si>
   <si>
+    <t>Henry</t>
+  </si>
+  <si>
+    <t>UPC000052</t>
+  </si>
+  <si>
     <t>Hoang</t>
-  </si>
-  <si>
-    <t>UPC000052</t>
-  </si>
-  <si>
-    <t>Henry</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <sz val="11.0"/>
@@ -373,11 +353,11 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <sz val="12.0"/>
+      <sz val="14.0"/>
       <b val="true"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -392,16 +372,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor indexed="22"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="none">
-        <fgColor indexed="52"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="52"/>
       </patternFill>
     </fill>
   </fills>
@@ -435,7 +405,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="center"/>
@@ -444,24 +414,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="true" applyNumberFormat="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyBorder="true" applyFill="true" applyAlignment="true">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="true" applyNumberFormat="true"/>
   </cellXfs>
 </styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="9.96484375" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="53.453125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="9.03515625" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="8.71875" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="7.40234375" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="10.54296875" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="10.171875" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="6.40234375" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -492,10 +459,10 @@
         <v>7</v>
       </c>
       <c r="D2" t="n" s="3">
-        <v>22.0</v>
+        <v>88.0</v>
       </c>
       <c r="E2" t="n" s="4">
-        <v>93.99</v>
+        <v>100.91</v>
       </c>
     </row>
     <row r="3">
@@ -509,7 +476,7 @@
         <v>7</v>
       </c>
       <c r="D3" t="n" s="3">
-        <v>44.0</v>
+        <v>39.0</v>
       </c>
       <c r="E3" t="n" s="4">
         <v>88.99</v>
@@ -526,7 +493,7 @@
         <v>7</v>
       </c>
       <c r="D4" t="n" s="3">
-        <v>40.0</v>
+        <v>39.0</v>
       </c>
       <c r="E4" t="n" s="4">
         <v>90.99</v>
@@ -543,7 +510,7 @@
         <v>7</v>
       </c>
       <c r="D5" t="n" s="3">
-        <v>30.0</v>
+        <v>18.0</v>
       </c>
       <c r="E5" t="n" s="4">
         <v>112.99</v>
@@ -560,7 +527,7 @@
         <v>7</v>
       </c>
       <c r="D6" t="n" s="3">
-        <v>60.0</v>
+        <v>59.0</v>
       </c>
       <c r="E6" t="n" s="4">
         <v>89.99</v>
@@ -611,7 +578,7 @@
         <v>22</v>
       </c>
       <c r="D9" t="n" s="3">
-        <v>45.0</v>
+        <v>46.0</v>
       </c>
       <c r="E9" t="n" s="4">
         <v>31.99</v>
@@ -645,7 +612,7 @@
         <v>22</v>
       </c>
       <c r="D11" t="n" s="3">
-        <v>50.0</v>
+        <v>49.0</v>
       </c>
       <c r="E11" t="n" s="4">
         <v>19.79</v>
@@ -849,7 +816,7 @@
         <v>7</v>
       </c>
       <c r="D23" t="n" s="3">
-        <v>20.0</v>
+        <v>19.0</v>
       </c>
       <c r="E23" t="n" s="4">
         <v>88.99</v>
@@ -866,10 +833,10 @@
         <v>7</v>
       </c>
       <c r="D24" t="n" s="3">
-        <v>25.0</v>
+        <v>30.0</v>
       </c>
       <c r="E24" t="n" s="4">
-        <v>29.99</v>
+        <v>36.99</v>
       </c>
     </row>
     <row r="25">
@@ -883,10 +850,10 @@
         <v>7</v>
       </c>
       <c r="D25" t="n" s="3">
-        <v>30.0</v>
+        <v>20.0</v>
       </c>
       <c r="E25" t="n" s="4">
-        <v>36.99</v>
+        <v>105.99</v>
       </c>
     </row>
     <row r="26">
@@ -900,10 +867,10 @@
         <v>7</v>
       </c>
       <c r="D26" t="n" s="3">
-        <v>20.0</v>
+        <v>60.0</v>
       </c>
       <c r="E26" t="n" s="4">
-        <v>105.99</v>
+        <v>42.99</v>
       </c>
     </row>
     <row r="27">
@@ -917,10 +884,10 @@
         <v>7</v>
       </c>
       <c r="D27" t="n" s="3">
-        <v>60.0</v>
+        <v>40.0</v>
       </c>
       <c r="E27" t="n" s="4">
-        <v>42.99</v>
+        <v>38.99</v>
       </c>
     </row>
     <row r="28">
@@ -934,10 +901,10 @@
         <v>7</v>
       </c>
       <c r="D28" t="n" s="3">
-        <v>40.0</v>
+        <v>100.0</v>
       </c>
       <c r="E28" t="n" s="4">
-        <v>38.99</v>
+        <v>5.19</v>
       </c>
     </row>
     <row r="29">
@@ -951,7 +918,7 @@
         <v>7</v>
       </c>
       <c r="D29" t="n" s="3">
-        <v>100.0</v>
+        <v>90.0</v>
       </c>
       <c r="E29" t="n" s="4">
         <v>5.19</v>
@@ -965,13 +932,13 @@
         <v>64</v>
       </c>
       <c r="C30" t="s" s="2">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="D30" t="n" s="3">
-        <v>90.0</v>
+        <v>45.0</v>
       </c>
       <c r="E30" t="n" s="4">
-        <v>5.19</v>
+        <v>38.99</v>
       </c>
     </row>
     <row r="31">
@@ -985,10 +952,10 @@
         <v>22</v>
       </c>
       <c r="D31" t="n" s="3">
-        <v>45.0</v>
+        <v>35.0</v>
       </c>
       <c r="E31" t="n" s="4">
-        <v>38.99</v>
+        <v>41.99</v>
       </c>
     </row>
     <row r="32">
@@ -1002,10 +969,10 @@
         <v>22</v>
       </c>
       <c r="D32" t="n" s="3">
-        <v>35.0</v>
+        <v>40.0</v>
       </c>
       <c r="E32" t="n" s="4">
-        <v>41.99</v>
+        <v>40.99</v>
       </c>
     </row>
     <row r="33">
@@ -1019,10 +986,10 @@
         <v>22</v>
       </c>
       <c r="D33" t="n" s="3">
-        <v>40.0</v>
+        <v>30.0</v>
       </c>
       <c r="E33" t="n" s="4">
-        <v>40.99</v>
+        <v>34.99</v>
       </c>
     </row>
     <row r="34">
@@ -1036,10 +1003,10 @@
         <v>22</v>
       </c>
       <c r="D34" t="n" s="3">
-        <v>30.0</v>
+        <v>25.0</v>
       </c>
       <c r="E34" t="n" s="4">
-        <v>34.99</v>
+        <v>30.99</v>
       </c>
     </row>
     <row r="35">
@@ -1050,30 +1017,30 @@
         <v>74</v>
       </c>
       <c r="C35" t="s" s="2">
-        <v>22</v>
+        <v>75</v>
       </c>
       <c r="D35" t="n" s="3">
-        <v>25.0</v>
+        <v>100.0</v>
       </c>
       <c r="E35" t="n" s="4">
-        <v>30.99</v>
+        <v>4.99</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="B36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="C36" t="s" s="2">
         <v>75</v>
       </c>
-      <c r="B36" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="C36" t="s" s="2">
-        <v>77</v>
-      </c>
       <c r="D36" t="n" s="3">
-        <v>100.0</v>
+        <v>80.0</v>
       </c>
       <c r="E36" t="n" s="4">
-        <v>4.99</v>
+        <v>29.99</v>
       </c>
     </row>
     <row r="37">
@@ -1084,30 +1051,30 @@
         <v>79</v>
       </c>
       <c r="C37" t="s" s="2">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D37" t="n" s="3">
-        <v>80.0</v>
+        <v>60.0</v>
       </c>
       <c r="E37" t="n" s="4">
-        <v>29.99</v>
+        <v>40.99</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C38" t="s" s="2">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="D38" t="n" s="3">
-        <v>60.0</v>
+        <v>50.0</v>
       </c>
       <c r="E38" t="n" s="4">
-        <v>40.99</v>
+        <v>17.49</v>
       </c>
     </row>
     <row r="39">
@@ -1118,13 +1085,13 @@
         <v>84</v>
       </c>
       <c r="C39" t="s" s="2">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D39" t="n" s="3">
-        <v>50.0</v>
+        <v>45.0</v>
       </c>
       <c r="E39" t="n" s="4">
-        <v>17.49</v>
+        <v>10.49</v>
       </c>
     </row>
     <row r="40">
@@ -1135,30 +1102,30 @@
         <v>86</v>
       </c>
       <c r="C40" t="s" s="2">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="D40" t="n" s="3">
-        <v>45.0</v>
+        <v>74.0</v>
       </c>
       <c r="E40" t="n" s="4">
-        <v>10.49</v>
+        <v>25.99</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="B41" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="C41" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="B41" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="C41" t="s" s="2">
-        <v>89</v>
-      </c>
       <c r="D41" t="n" s="3">
-        <v>75.0</v>
+        <v>90.0</v>
       </c>
       <c r="E41" t="n" s="4">
-        <v>25.99</v>
+        <v>14.99</v>
       </c>
     </row>
     <row r="42">
@@ -1169,13 +1136,13 @@
         <v>91</v>
       </c>
       <c r="C42" t="s" s="2">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D42" t="n" s="3">
-        <v>90.0</v>
+        <v>30.0</v>
       </c>
       <c r="E42" t="n" s="4">
-        <v>14.99</v>
+        <v>50.99</v>
       </c>
     </row>
     <row r="43">
@@ -1186,13 +1153,13 @@
         <v>93</v>
       </c>
       <c r="C43" t="s" s="2">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D43" t="n" s="3">
-        <v>30.0</v>
+        <v>40.0</v>
       </c>
       <c r="E43" t="n" s="4">
-        <v>50.99</v>
+        <v>44.99</v>
       </c>
     </row>
     <row r="44">
@@ -1203,13 +1170,13 @@
         <v>95</v>
       </c>
       <c r="C44" t="s" s="2">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D44" t="n" s="3">
-        <v>40.0</v>
+        <v>60.0</v>
       </c>
       <c r="E44" t="n" s="4">
-        <v>44.99</v>
+        <v>19.99</v>
       </c>
     </row>
     <row r="45">
@@ -1220,13 +1187,13 @@
         <v>97</v>
       </c>
       <c r="C45" t="s" s="2">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D45" t="n" s="3">
-        <v>60.0</v>
+        <v>49.0</v>
       </c>
       <c r="E45" t="n" s="4">
-        <v>19.99</v>
+        <v>39.99</v>
       </c>
     </row>
     <row r="46">
@@ -1237,13 +1204,13 @@
         <v>99</v>
       </c>
       <c r="C46" t="s" s="2">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D46" t="n" s="3">
-        <v>50.0</v>
+        <v>70.0</v>
       </c>
       <c r="E46" t="n" s="4">
-        <v>39.99</v>
+        <v>24.99</v>
       </c>
     </row>
     <row r="47">
@@ -1254,13 +1221,13 @@
         <v>101</v>
       </c>
       <c r="C47" t="s" s="2">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D47" t="n" s="3">
-        <v>70.0</v>
+        <v>100.0</v>
       </c>
       <c r="E47" t="n" s="4">
-        <v>24.99</v>
+        <v>12.99</v>
       </c>
     </row>
     <row r="48">
@@ -1271,13 +1238,13 @@
         <v>103</v>
       </c>
       <c r="C48" t="s" s="2">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="D48" t="n" s="3">
-        <v>100.0</v>
+        <v>10.0</v>
       </c>
       <c r="E48" t="n" s="4">
-        <v>12.99</v>
+        <v>9.99</v>
       </c>
     </row>
     <row r="49">
@@ -1288,13 +1255,13 @@
         <v>105</v>
       </c>
       <c r="C49" t="s" s="2">
-        <v>7</v>
+        <v>75</v>
       </c>
       <c r="D49" t="n" s="3">
-        <v>40.0</v>
+        <v>21.0</v>
       </c>
       <c r="E49" t="n" s="4">
-        <v>82.49</v>
+        <v>9.99</v>
       </c>
     </row>
     <row r="50">
@@ -1305,63 +1272,12 @@
         <v>107</v>
       </c>
       <c r="C50" t="s" s="2">
-        <v>22</v>
+        <v>80</v>
       </c>
       <c r="D50" t="n" s="3">
-        <v>50.0</v>
+        <v>1.0</v>
       </c>
       <c r="E50" t="n" s="4">
-        <v>68.99</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="s" s="2">
-        <v>108</v>
-      </c>
-      <c r="B51" t="s" s="2">
-        <v>109</v>
-      </c>
-      <c r="C51" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="D51" t="n" s="3">
-        <v>120.0</v>
-      </c>
-      <c r="E51" t="n" s="4">
-        <v>9.99</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="s" s="5">
-        <v>110</v>
-      </c>
-      <c r="B52" t="s" s="5">
-        <v>111</v>
-      </c>
-      <c r="C52" t="s" s="5">
-        <v>22</v>
-      </c>
-      <c r="D52" t="n" s="5">
-        <v>10.0</v>
-      </c>
-      <c r="E52" t="n" s="5">
-        <v>100.0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="s" s="5">
-        <v>112</v>
-      </c>
-      <c r="B53" t="s" s="5">
-        <v>113</v>
-      </c>
-      <c r="C53" t="s" s="5">
-        <v>89</v>
-      </c>
-      <c r="D53" t="n" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="E53" t="n" s="5">
         <v>100.0</v>
       </c>
     </row>

</xml_diff>